<commit_message>
update a la db
</commit_message>
<xml_diff>
--- a/db/Diccionario_de_datos_TourismEasy.xlsx
+++ b/db/Diccionario_de_datos_TourismEasy.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F342"/>
+  <dimension ref="A1:F343"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2377,7 +2377,7 @@
         </is>
       </c>
     </row>
-    <row r="83" ht="32" customHeight="1">
+    <row r="83" ht="45.5" customHeight="1">
       <c r="A83" s="5" t="inlineStr">
         <is>
           <t>ID_PERSONA_ECOMMERCE</t>
@@ -2405,7 +2405,8 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>HISTORIAL_CONTRASENAS_USUARIO_ECOMMERCE</t>
+          <t>HISTORIAL_CONTRASENAS_USUARIO_ECOMMERCE
+TOKENS_RECUPERACION</t>
         </is>
       </c>
     </row>
@@ -3214,7 +3215,7 @@
       </c>
       <c r="B122" s="5" t="inlineStr">
         <is>
-          <t>SERIAL</t>
+          <t>DECIMAL(10,0)</t>
         </is>
       </c>
       <c r="C122" s="6" t="inlineStr">
@@ -3352,7 +3353,7 @@
       </c>
       <c r="D126" s="5" t="inlineStr">
         <is>
-          <t>Fecha de salida (no puede ser anterior a la fecha actual).</t>
+          <t>Fecha de salida del servicio de transporte.</t>
         </is>
       </c>
       <c r="E126" s="7" t="inlineStr">
@@ -3674,7 +3675,7 @@
       </c>
       <c r="B139" s="5" t="inlineStr">
         <is>
-          <t>SERIAL</t>
+          <t>DECIMAL(10,0)</t>
         </is>
       </c>
       <c r="C139" s="6" t="inlineStr">
@@ -3846,7 +3847,7 @@
       </c>
       <c r="B147" s="5" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>DECIMAL(10,0)</t>
         </is>
       </c>
       <c r="C147" s="6" t="inlineStr">
@@ -3878,7 +3879,7 @@
       </c>
       <c r="B148" s="5" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>DECIMAL(10,0)</t>
         </is>
       </c>
       <c r="C148" s="6" t="inlineStr">
@@ -3954,7 +3955,7 @@
       </c>
       <c r="B153" s="5" t="inlineStr">
         <is>
-          <t>SERIAL</t>
+          <t>DECIMAL(10,0)</t>
         </is>
       </c>
       <c r="C153" s="6" t="inlineStr">
@@ -4126,7 +4127,7 @@
       </c>
       <c r="B161" s="5" t="inlineStr">
         <is>
-          <t>SERIAL</t>
+          <t>DECIMAL(10,0)</t>
         </is>
       </c>
       <c r="C161" s="6" t="inlineStr">
@@ -4619,7 +4620,7 @@
       </c>
       <c r="B179" s="5" t="inlineStr">
         <is>
-          <t>SERIAL</t>
+          <t>DECIMAL(10,0)</t>
         </is>
       </c>
       <c r="C179" s="6" t="inlineStr">
@@ -5143,7 +5144,7 @@
       </c>
       <c r="B198" s="5" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>DECIMAL(10,0)</t>
         </is>
       </c>
       <c r="C198" s="6" t="inlineStr">
@@ -5175,7 +5176,7 @@
       </c>
       <c r="B199" s="5" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>DECIMAL(10,0)</t>
         </is>
       </c>
       <c r="C199" s="6" t="inlineStr">
@@ -5283,7 +5284,7 @@
       </c>
       <c r="B205" s="5" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>DECIMAL(10,0)</t>
         </is>
       </c>
       <c r="C205" s="6" t="inlineStr">
@@ -5347,7 +5348,7 @@
       </c>
       <c r="B207" s="5" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>DECIMAL(10,0)</t>
         </is>
       </c>
       <c r="C207" s="6" t="inlineStr">
@@ -5455,7 +5456,7 @@
       </c>
       <c r="B213" s="5" t="inlineStr">
         <is>
-          <t>SERIAL</t>
+          <t>DECIMAL(10,0)</t>
         </is>
       </c>
       <c r="C213" s="6" t="inlineStr">
@@ -8319,7 +8320,7 @@
         </is>
       </c>
     </row>
-    <row r="329" ht="18.5" customHeight="1">
+    <row r="329" ht="45.5" customHeight="1">
       <c r="A329" s="5" t="inlineStr">
         <is>
           <t>ID_USUARIO</t>
@@ -8337,7 +8338,7 @@
       </c>
       <c r="D329" s="5" t="inlineStr">
         <is>
-          <t>Usuario que solicita la recuperación (si aplica).</t>
+          <t>Usuario administrador que solicita la recuperación (si aplica). Exactamente uno de los tres (ID_USUARIO, ID_EMPRESA o ID_PERSONA_ECOMMERCE) debe estar lleno.</t>
         </is>
       </c>
       <c r="E329" s="5" t="inlineStr">
@@ -8351,7 +8352,7 @@
         </is>
       </c>
     </row>
-    <row r="330" ht="18.5" customHeight="1">
+    <row r="330" ht="45.5" customHeight="1">
       <c r="A330" s="5" t="inlineStr">
         <is>
           <t>ID_EMPRESA</t>
@@ -8369,7 +8370,7 @@
       </c>
       <c r="D330" s="5" t="inlineStr">
         <is>
-          <t>Cuenta de empresa que solicita la recuperación (si aplica).</t>
+          <t>Cuenta de empresa que solicita la recuperación (si aplica). Exactamente uno de los tres (ID_USUARIO, ID_EMPRESA o ID_PERSONA_ECOMMERCE) debe estar lleno.</t>
         </is>
       </c>
       <c r="E330" s="5" t="inlineStr">
@@ -8383,57 +8384,57 @@
         </is>
       </c>
     </row>
-    <row r="331" ht="32" customHeight="1">
+    <row r="331" ht="45.5" customHeight="1">
       <c r="A331" s="5" t="inlineStr">
         <is>
+          <t>ID_PERSONA_ECOMMERCE</t>
+        </is>
+      </c>
+      <c r="B331" s="5" t="inlineStr">
+        <is>
+          <t>VARCHAR(10)</t>
+        </is>
+      </c>
+      <c r="C331" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D331" s="5" t="inlineStr">
+        <is>
+          <t>Usuario del e-commerce que solicita la recuperación (si aplica). Exactamente uno de los tres (ID_USUARIO, ID_EMPRESA o ID_PERSONA_ECOMMERCE) debe estar lleno.</t>
+        </is>
+      </c>
+      <c r="E331" s="5" t="inlineStr">
+        <is>
+          <t>USUARIOS_ECOMMERCE</t>
+        </is>
+      </c>
+      <c r="F331" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="332" ht="32" customHeight="1">
+      <c r="A332" s="5" t="inlineStr">
+        <is>
           <t>TOKEN</t>
         </is>
       </c>
-      <c r="B331" s="5" t="inlineStr">
+      <c r="B332" s="5" t="inlineStr">
         <is>
           <t>VARCHAR(64)</t>
         </is>
       </c>
-      <c r="C331" s="6" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="D331" s="5" t="inlineStr">
+      <c r="C332" s="6" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D332" s="5" t="inlineStr">
         <is>
           <t>Token de recuperación de 64 caracteres hexadecimales (valor único).</t>
-        </is>
-      </c>
-      <c r="E331" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F331" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="332" ht="18.5" customHeight="1">
-      <c r="A332" s="5" t="inlineStr">
-        <is>
-          <t>FECHA_CREACION</t>
-        </is>
-      </c>
-      <c r="B332" s="5" t="inlineStr">
-        <is>
-          <t>TIMESTAMP</t>
-        </is>
-      </c>
-      <c r="C332" s="6" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="D332" s="5" t="inlineStr">
-        <is>
-          <t>Fecha y hora de creación del token.</t>
         </is>
       </c>
       <c r="E332" s="7" t="inlineStr">
@@ -8450,7 +8451,7 @@
     <row r="333" ht="18.5" customHeight="1">
       <c r="A333" s="5" t="inlineStr">
         <is>
-          <t>FECHA_EXPIRA</t>
+          <t>FECHA_CREACION</t>
         </is>
       </c>
       <c r="B333" s="5" t="inlineStr">
@@ -8465,7 +8466,7 @@
       </c>
       <c r="D333" s="5" t="inlineStr">
         <is>
-          <t>Fecha y hora de expiración (posterior a la creación).</t>
+          <t>Fecha y hora de creación del token.</t>
         </is>
       </c>
       <c r="E333" s="7" t="inlineStr">
@@ -8482,167 +8483,167 @@
     <row r="334" ht="18.5" customHeight="1">
       <c r="A334" s="5" t="inlineStr">
         <is>
+          <t>FECHA_EXPIRA</t>
+        </is>
+      </c>
+      <c r="B334" s="5" t="inlineStr">
+        <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="C334" s="6" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D334" s="5" t="inlineStr">
+        <is>
+          <t>Fecha y hora de expiración (posterior a la creación).</t>
+        </is>
+      </c>
+      <c r="E334" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F334" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="335" ht="18.5" customHeight="1">
+      <c r="A335" s="5" t="inlineStr">
+        <is>
           <t>USADO</t>
         </is>
       </c>
-      <c r="B334" s="5" t="inlineStr">
+      <c r="B335" s="5" t="inlineStr">
         <is>
           <t>BOOLEAN</t>
         </is>
       </c>
-      <c r="C334" s="6" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="D334" s="5" t="inlineStr">
+      <c r="C335" s="6" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D335" s="5" t="inlineStr">
         <is>
           <t>Indica si el token ya fue utilizado (por defecto FALSE).</t>
         </is>
       </c>
-      <c r="E334" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F334" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="337" ht="21" customHeight="1">
-      <c r="A337" s="2" t="inlineStr">
+      <c r="E335" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F335" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="338" ht="21" customHeight="1">
+      <c r="A338" s="2" t="inlineStr">
         <is>
           <t>TABLA 33: LIKES_RESENAS</t>
         </is>
       </c>
-      <c r="B337" s="3" t="n"/>
-      <c r="C337" s="3" t="n"/>
-      <c r="D337" s="3" t="n"/>
-      <c r="E337" s="3" t="n"/>
-      <c r="F337" s="3" t="n"/>
-    </row>
-    <row r="338" ht="30" customHeight="1">
-      <c r="A338" s="4" t="inlineStr">
+      <c r="B338" s="3" t="n"/>
+      <c r="C338" s="3" t="n"/>
+      <c r="D338" s="3" t="n"/>
+      <c r="E338" s="3" t="n"/>
+      <c r="F338" s="3" t="n"/>
+    </row>
+    <row r="339" ht="30" customHeight="1">
+      <c r="A339" s="4" t="inlineStr">
         <is>
           <t>Atributo</t>
         </is>
       </c>
-      <c r="B338" s="4" t="inlineStr">
+      <c r="B339" s="4" t="inlineStr">
         <is>
           <t>Tipo de dato</t>
         </is>
       </c>
-      <c r="C338" s="4" t="inlineStr">
+      <c r="C339" s="4" t="inlineStr">
         <is>
           <t>Restricción (¿NOT NULL?)</t>
         </is>
       </c>
-      <c r="D338" s="4" t="inlineStr">
+      <c r="D339" s="4" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="E338" s="4" t="inlineStr">
+      <c r="E339" s="4" t="inlineStr">
         <is>
           <t>Tabla referida</t>
         </is>
       </c>
-      <c r="F338" s="4" t="inlineStr">
+      <c r="F339" s="4" t="inlineStr">
         <is>
           <t>Tabla referente</t>
         </is>
       </c>
     </row>
-    <row r="339" ht="18.5" customHeight="1">
-      <c r="A339" s="5" t="inlineStr">
+    <row r="340" ht="18.5" customHeight="1">
+      <c r="A340" s="5" t="inlineStr">
         <is>
           <t>ID_LIKE</t>
         </is>
       </c>
-      <c r="B339" s="5" t="inlineStr">
+      <c r="B340" s="5" t="inlineStr">
         <is>
           <t>SERIAL</t>
         </is>
       </c>
-      <c r="C339" s="6" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="D339" s="5" t="inlineStr">
+      <c r="C340" s="6" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D340" s="5" t="inlineStr">
         <is>
           <t>Llave primaria. Identificador autoincremental del like.</t>
         </is>
       </c>
-      <c r="E339" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F339" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="340" ht="32" customHeight="1">
-      <c r="A340" s="5" t="inlineStr">
+      <c r="E340" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F340" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="341" ht="32" customHeight="1">
+      <c r="A341" s="5" t="inlineStr">
         <is>
           <t>ID_RESENA</t>
         </is>
       </c>
-      <c r="B340" s="5" t="inlineStr">
-        <is>
-          <t>INT</t>
-        </is>
-      </c>
-      <c r="C340" s="6" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="D340" s="5" t="inlineStr">
+      <c r="B341" s="5" t="inlineStr">
+        <is>
+          <t>DECIMAL(10,0)</t>
+        </is>
+      </c>
+      <c r="C341" s="6" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D341" s="5" t="inlineStr">
         <is>
           <t>Reseña a la que se da el like (un like por visitante en cada reseña).</t>
         </is>
       </c>
-      <c r="E340" s="5" t="inlineStr">
+      <c r="E341" s="5" t="inlineStr">
         <is>
           <t>RESENAS_PLATAFORMA</t>
-        </is>
-      </c>
-      <c r="F340" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="341" ht="18.5" customHeight="1">
-      <c r="A341" s="5" t="inlineStr">
-        <is>
-          <t>VISITOR_ID</t>
-        </is>
-      </c>
-      <c r="B341" s="5" t="inlineStr">
-        <is>
-          <t>VARCHAR(64)</t>
-        </is>
-      </c>
-      <c r="C341" s="6" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="D341" s="5" t="inlineStr">
-        <is>
-          <t>Identificador anónimo del visitante (10 a 64 caracteres).</t>
-        </is>
-      </c>
-      <c r="E341" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
         </is>
       </c>
       <c r="F341" s="7" t="inlineStr">
@@ -8654,30 +8655,62 @@
     <row r="342" ht="18.5" customHeight="1">
       <c r="A342" s="5" t="inlineStr">
         <is>
+          <t>VISITOR_ID</t>
+        </is>
+      </c>
+      <c r="B342" s="5" t="inlineStr">
+        <is>
+          <t>VARCHAR(64)</t>
+        </is>
+      </c>
+      <c r="C342" s="6" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D342" s="5" t="inlineStr">
+        <is>
+          <t>Identificador anónimo del visitante (10 a 64 caracteres).</t>
+        </is>
+      </c>
+      <c r="E342" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F342" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="343" ht="18.5" customHeight="1">
+      <c r="A343" s="5" t="inlineStr">
+        <is>
           <t>FECHA_LIKE</t>
         </is>
       </c>
-      <c r="B342" s="5" t="inlineStr">
+      <c r="B343" s="5" t="inlineStr">
         <is>
           <t>TIMESTAMP</t>
         </is>
       </c>
-      <c r="C342" s="6" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="D342" s="5" t="inlineStr">
+      <c r="C343" s="6" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D343" s="5" t="inlineStr">
         <is>
           <t>Fecha y hora del like.</t>
         </is>
       </c>
-      <c r="E342" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F342" s="7" t="inlineStr">
+      <c r="E343" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F343" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -8710,8 +8743,8 @@
     <mergeCell ref="A220:F220"/>
     <mergeCell ref="A258:F258"/>
     <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A338:F338"/>
     <mergeCell ref="A114:F114"/>
-    <mergeCell ref="A337:F337"/>
     <mergeCell ref="A226:F226"/>
     <mergeCell ref="A284:F284"/>
     <mergeCell ref="A296:F296"/>

</xml_diff>